<commit_message>
Combine filters and add local logo storage
</commit_message>
<xml_diff>
--- a/data/PPDB database.xlsx
+++ b/data/PPDB database.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PPDB" sheetId="1" r:id="R6bda48bb4a7441c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PPDB" sheetId="1" r:id="Rd092780b579f4c26"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -172,14 +172,16 @@
     <x:r>
       <x:rPr>
         <x:b/>
-        <x:color theme="1"/>
+        <x:sz val="1000"/>
+        <x:color rgb="FF000000"/>
         <x:rFont val="Arial"/>
       </x:rPr>
       <x:t xml:space="preserve">The new People's Party</x:t>
     </x:r>
     <x:r>
       <x:rPr>
-        <x:color theme="1"/>
+        <x:sz val="1000"/>
+        <x:color rgb="FF000000"/>
         <x:rFont val="Arial"/>
       </x:rPr>
       <x:t xml:space="preserve"> (</x:t>
@@ -187,14 +189,16 @@
     <x:r>
       <x:rPr>
         <x:i/>
-        <x:color theme="1"/>
+        <x:sz val="1000"/>
+        <x:color rgb="FF000000"/>
         <x:rFont val="Arial"/>
       </x:rPr>
       <x:t xml:space="preserve">Die neue Volkspartei</x:t>
     </x:r>
     <x:r>
       <x:rPr>
-        <x:color theme="1"/>
+        <x:sz val="1000"/>
+        <x:color rgb="FF000000"/>
         <x:rFont val="Arial"/>
       </x:rPr>
       <x:t xml:space="preserve">, 2017-2022, unofficial)</x:t>
@@ -283,14 +287,16 @@
     <x:r>
       <x:rPr>
         <x:b/>
-        <x:color theme="1"/>
+        <x:sz val="1000"/>
+        <x:color rgb="FF000000"/>
         <x:rFont val="Arial"/>
       </x:rPr>
       <x:t xml:space="preserve">Communist Party of Lithuania (Independent)</x:t>
     </x:r>
     <x:r>
       <x:rPr>
-        <x:color theme="1"/>
+        <x:sz val="1000"/>
+        <x:color rgb="FF000000"/>
         <x:rFont val="Arial"/>
       </x:rPr>
       <x:t xml:space="preserve"> (</x:t>
@@ -298,14 +304,16 @@
     <x:r>
       <x:rPr>
         <x:i/>
-        <x:color theme="1"/>
+        <x:sz val="1000"/>
+        <x:color rgb="FF000000"/>
         <x:rFont val="Arial"/>
       </x:rPr>
       <x:t xml:space="preserve">Lietuvos komunistų partija (nepriklausoma)</x:t>
     </x:r>
     <x:r>
       <x:rPr>
-        <x:color theme="1"/>
+        <x:sz val="1000"/>
+        <x:color rgb="FF000000"/>
         <x:rFont val="Arial"/>
       </x:rPr>
       <x:t xml:space="preserve">, until 1990)</x:t>
@@ -936,7 +944,7 @@
         <x:v>6.0</x:v>
       </x:c>
       <x:c r="I4" s="5" t="str">
-        <x:v>https://upload.wikimedia.org/wikipedia/commons/thumb/0/01/Logo_of_the_Freedom_Party_of_Austria.svg/330px-Logo_of_the_Freedom_Party_of_Austria.svg.png</x:v>
+        <x:v>/media/logos/atFPO.png</x:v>
       </x:c>
       <x:c r="J4" s="6" t="str">
         <x:v>#005EA8</x:v>
@@ -1329,15 +1337,15 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="R87cbc89e22554d33"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T3" r:id="R9e73267f78824d3e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V3" r:id="Re4ae21b23ba64ce1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE3" r:id="R840d85b5d3d549e4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="R2875397e568b43b1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T4" r:id="R56d05ec92b5c4677"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE4" r:id="Rd8644673fc2f4686"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="R6a4f66d0a2914693"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE5" r:id="R544c222c7039427a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="R3a9b70bae0464f93"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T3" r:id="Rf8441ef41d8f481a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V3" r:id="Re550199c8cee4037"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE3" r:id="R6e45390becd241e9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="R7314c4180e99426b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T4" r:id="Rc8c277f459af4920"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE4" r:id="Rbde6f0f3eee94e0f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="R5469210bfa734226"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE5" r:id="Rc41aeca45a3a4abe"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Add PPDB branding and legislature representation
</commit_message>
<xml_diff>
--- a/data/PPDB database.xlsx
+++ b/data/PPDB database.xlsx
@@ -2,7 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PPDB" sheetId="1" r:id="Rd092780b579f4c26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PPDB" sheetId="1" r:id="Rcc34046a6fd14c9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legislatures" sheetId="2" r:id="Re2e7b0d92750461b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -342,11 +343,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
+  <x:numFmts count="3">
     <x:numFmt numFmtId="164" formatCode="dd-mm-yyyy"/>
     <x:numFmt numFmtId="165" formatCode="d-m-yyyy"/>
+    <x:numFmt numFmtId="200" formatCode="#,##0"/>
   </x:numFmts>
-  <x:fonts count="11">
+  <x:fonts count="13">
     <x:font>
       <x:sz val="10"/>
       <x:color rgb="FF000000"/>
@@ -394,8 +396,20 @@
       <x:color theme="1"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF333333"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -412,14 +426,43 @@
         <x:fgColor rgb="FFF8F9FA"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD8D8D8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF08057F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEEEEEE"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="1">
+  <x:borders count="2">
     <x:border/>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FF777777"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FF777777"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF777777"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF777777"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyAlignment="1"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="17">
+  <x:cellXfs count="26">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment vertical="bottom" wrapText="0"/>
     </x:xf>
@@ -445,11 +488,50 @@
       <x:alignment horizontal="right" vertical="bottom"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="0"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
 </x:styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LegislaturesTable" displayName="LegislaturesTable" ref="A2:D3" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="4">
+    <x:tableColumn id="1" name="COUNTRY"/>
+    <x:tableColumn id="2" name="LOWER_HOUSE_TOTAL"/>
+    <x:tableColumn id="3" name="UPPER_HOUSE_TOTAL"/>
+    <x:tableColumn id="4" name="MEP_TOTAL"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -940,8 +1022,8 @@
       <x:c r="G4" s="1">
         <x:v>16.0</x:v>
       </x:c>
-      <x:c r="H4" s="1">
-        <x:v>6.0</x:v>
+      <x:c r="H4" s="1" t="n">
+        <x:v>5</x:v>
       </x:c>
       <x:c r="I4" s="5" t="str">
         <x:v>/media/logos/atFPO.png</x:v>
@@ -1337,16 +1419,76 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="R3a9b70bae0464f93"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T3" r:id="Rf8441ef41d8f481a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V3" r:id="Re550199c8cee4037"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE3" r:id="R6e45390becd241e9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="R7314c4180e99426b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T4" r:id="Rc8c277f459af4920"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE4" r:id="Rbde6f0f3eee94e0f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="R5469210bfa734226"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE5" r:id="Rc41aeca45a3a4abe"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="Rbb593f92c8b5478b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T3" r:id="Rcac9be316af941a2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V3" r:id="R10ae5b0d1eb14f89"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE3" r:id="R3abed831212043ea"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="Rcf2dee0391c9499c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T4" r:id="R04bfe81114a543b2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE4" r:id="R9b033a8409a74078"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="R9816871d09d44bfe"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE5" r:id="Rb9ffe896944240f7"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="19" t="str">
+        <x:v>Text</x:v>
+      </x:c>
+      <x:c r="B1" s="19" t="str">
+        <x:v>Parameter</x:v>
+      </x:c>
+      <x:c r="C1" s="19" t="str">
+        <x:v>Parameter</x:v>
+      </x:c>
+      <x:c r="D1" s="19" t="str">
+        <x:v>Parameter</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="22" t="str">
+        <x:v>COUNTRY</x:v>
+      </x:c>
+      <x:c r="B2" s="22" t="str">
+        <x:v>LOWER_HOUSE_TOTAL</x:v>
+      </x:c>
+      <x:c r="C2" s="22" t="str">
+        <x:v>UPPER_HOUSE_TOTAL</x:v>
+      </x:c>
+      <x:c r="D2" s="22" t="str">
+        <x:v>MEP_TOTAL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="24" t="str">
+        <x:v>Austria</x:v>
+      </x:c>
+      <x:c r="B3" s="25" t="n">
+        <x:v>183</x:v>
+      </x:c>
+      <x:c r="C3" s="25" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="D3" s="25" t="n">
+        <x:v>20</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95352c4993e04756"/>
+  </x:tableParts>
+</x:worksheet>
 </file>
</xml_diff>